<commit_message>
PCB update PG -40min
</commit_message>
<xml_diff>
--- a/Dokumentation/Arbeitszeit.xlsx
+++ b/Dokumentation/Arbeitszeit.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Watzek\Documents\Diplom_Arbeit\Dokumentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEAA12EE-1A51-4E19-9E6B-C4182B868AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F25E6C-C62F-46C7-A7D2-CC372300639F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{22DE24AD-4B2B-4184-88E5-3CA953AB6CDD}"/>
+    <workbookView xWindow="3732" yWindow="3732" windowWidth="23040" windowHeight="12120" xr2:uid="{22DE24AD-4B2B-4184-88E5-3CA953AB6CDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -214,13 +214,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -568,16 +566,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -590,7 +588,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(B4:B23)</f>
-        <v>0.5</v>
+        <v>70</v>
       </c>
       <c r="C3" s="1">
         <f t="shared" ref="C3:E3" si="0">SUM(C4:C23)</f>
@@ -606,150 +604,135 @@
       </c>
       <c r="F3" s="1">
         <f>AVERAGE(B3:E3)</f>
-        <v>0.125</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="10"/>
+      <c r="B4" s="8">
+        <v>30</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="11"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="11"/>
+      <c r="B5" s="9">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="11"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="11"/>
+      <c r="B6" s="9">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="11"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="11"/>
+      <c r="B7" s="9"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="11"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="11"/>
+      <c r="B8" s="9"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="11"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="11"/>
+      <c r="B9" s="9"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="11"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="11"/>
+      <c r="B10" s="9"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="11"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="11"/>
+      <c r="B11" s="9"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="11"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="11"/>
+      <c r="B12" s="9"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="11"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="11"/>
+      <c r="B13" s="9"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="11"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="11"/>
+      <c r="B14" s="9"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="11"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="11"/>
+      <c r="B15" s="9"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="11"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="11"/>
+      <c r="B16" s="9"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="11"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="11"/>
+      <c r="B17" s="9"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="11"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="11"/>
+      <c r="B18" s="9"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="11"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="11"/>
+      <c r="B19" s="9"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="11"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="11"/>
+      <c r="B20" s="9"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="9"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="11"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="11"/>
+      <c r="B21" s="9"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="9"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="11"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="11"/>
+      <c r="B22" s="9"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="9"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="12"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="12"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
stressen und messure -30min
</commit_message>
<xml_diff>
--- a/Dokumentation/Arbeitszeit.xlsx
+++ b/Dokumentation/Arbeitszeit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F0D869-2DE5-4A0A-BA6C-83C3BAA3E0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB65E2C4-86B5-48B3-8CF0-D2E7FAEF5F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3732" yWindow="3732" windowWidth="23040" windowHeight="12120" xr2:uid="{22DE24AD-4B2B-4184-88E5-3CA953AB6CDD}"/>
   </bookViews>
@@ -588,7 +588,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(B4:B23)</f>
-        <v>230</v>
+        <v>295</v>
       </c>
       <c r="C3" s="1">
         <f t="shared" ref="C3:E3" si="0">SUM(C4:C23)</f>
@@ -604,7 +604,7 @@
       </c>
       <c r="F3" s="1">
         <f>AVERAGE(B3:E3)</f>
-        <v>57.5</v>
+        <v>73.75</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -657,7 +657,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" s="9">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -672,13 +672,17 @@
       <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="9"/>
+      <c r="B12" s="9">
+        <v>30</v>
+      </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="9"/>
+      <c r="B13" s="9">
+        <v>30</v>
+      </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="9"/>

</xml_diff>

<commit_message>
pcb und tuangabe überarbeitung -2h
</commit_message>
<xml_diff>
--- a/Dokumentation/Arbeitszeit.xlsx
+++ b/Dokumentation/Arbeitszeit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB65E2C4-86B5-48B3-8CF0-D2E7FAEF5F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B2E0E43-F2A7-471A-95C4-89F5E7231FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3732" yWindow="3732" windowWidth="23040" windowHeight="12120" xr2:uid="{22DE24AD-4B2B-4184-88E5-3CA953AB6CDD}"/>
   </bookViews>
@@ -60,6 +60,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -77,7 +80,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -210,11 +213,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -227,6 +241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -561,11 +576,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29C8FD97-DBFF-4488-882C-C2EA237EE42F}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -582,17 +600,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1">
         <f>SUM(B4:B23)</f>
-        <v>295</v>
+        <v>440</v>
       </c>
       <c r="C3" s="1">
         <f t="shared" ref="C3:E3" si="0">SUM(C4:C23)</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="D3" s="1">
         <f t="shared" si="0"/>
@@ -600,22 +618,31 @@
       </c>
       <c r="E3" s="1">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F3" s="1">
         <f>AVERAGE(B3:E3)</f>
-        <v>73.75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>148.75</v>
+      </c>
+      <c r="G3" s="12">
+        <f>F3/60</f>
+        <v>2.4791666666666665</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B4" s="8">
         <v>30</v>
       </c>
+      <c r="C4">
+        <v>75</v>
+      </c>
       <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
+      <c r="E4" s="11">
+        <v>80</v>
+      </c>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B5" s="9">
         <v>30</v>
       </c>
@@ -623,7 +650,7 @@
       <c r="E5" s="3"/>
       <c r="F5" s="9"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" s="9">
         <v>10</v>
       </c>
@@ -631,7 +658,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B7" s="9">
         <v>40</v>
       </c>
@@ -639,7 +666,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B8" s="9">
         <v>15</v>
       </c>
@@ -647,7 +674,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B9" s="9">
         <v>60</v>
       </c>
@@ -655,7 +682,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B10" s="9">
         <v>20</v>
       </c>
@@ -663,7 +690,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B11" s="9">
         <v>30</v>
       </c>
@@ -671,7 +698,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>30</v>
       </c>
@@ -679,7 +706,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B13" s="9">
         <v>30</v>
       </c>
@@ -687,26 +714,34 @@
       <c r="E13" s="3"/>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="9"/>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="9">
+        <v>45</v>
+      </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="9"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="9"/>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B15" s="9">
+        <v>10</v>
+      </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="9"/>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B16" s="9">
+        <v>60</v>
+      </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="9"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="9"/>
+      <c r="B17" s="9">
+        <v>30</v>
+      </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="9"/>

</xml_diff>